<commit_message>
screener: relatório de 2026-08-07
</commit_message>
<xml_diff>
--- a/reports/screener_2026-08-07.xlsx
+++ b/reports/screener_2026-08-07.xlsx
@@ -2318,7 +2318,7 @@
         <v>-14.1804789183963</v>
       </c>
       <c r="BS8" t="n">
-        <v>-41.3906633420233</v>
+        <v>-41.39066698170934</v>
       </c>
       <c r="BT8" t="b">
         <v>1</v>
@@ -5082,7 +5082,7 @@
         <v>-3.049647471931205</v>
       </c>
       <c r="BS20" t="n">
-        <v>-21.08023573257425</v>
+        <v>-21.08022686888683</v>
       </c>
       <c r="BT20" t="b">
         <v>1</v>
@@ -5771,7 +5771,7 @@
         <v>-3.496970464635651</v>
       </c>
       <c r="BS23" t="n">
-        <v>-18.64655512043243</v>
+        <v>-18.64656395665553</v>
       </c>
       <c r="BT23" t="b">
         <v>1</v>
@@ -12330,7 +12330,7 @@
         <v>9.15</v>
       </c>
       <c r="AQ52" t="n">
-        <v>8.710000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="AR52" t="n">
         <v>14.13</v>
@@ -12351,13 +12351,13 @@
         <v>15.75</v>
       </c>
       <c r="AZ52" t="n">
-        <v>9.800000000000001</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="BA52" t="n">
-        <v>18.16</v>
+        <v>18.15</v>
       </c>
       <c r="BB52" t="n">
-        <v>31.55</v>
+        <v>31.57</v>
       </c>
       <c r="BC52" t="n">
         <v>30.13</v>
@@ -12366,22 +12366,22 @@
         <v>35.04</v>
       </c>
       <c r="BE52" t="n">
-        <v>19.84</v>
+        <v>19.83</v>
       </c>
       <c r="BF52" t="n">
-        <v>18.16</v>
+        <v>18.15</v>
       </c>
       <c r="BG52" t="n">
-        <v>16.35</v>
+        <v>16.33</v>
       </c>
       <c r="BH52" t="n">
         <v>3</v>
       </c>
       <c r="BI52" t="n">
-        <v>3.8</v>
+        <v>3.69</v>
       </c>
       <c r="BJ52" t="n">
-        <v>25.96</v>
+        <v>25.92</v>
       </c>
       <c r="BK52" t="inlineStr">
         <is>
@@ -12406,13 +12406,13 @@
         </is>
       </c>
       <c r="BQ52" t="n">
-        <v>16.50235748291016</v>
+        <v>16.50238800048828</v>
       </c>
       <c r="BR52" t="n">
-        <v>-4.559090928004061</v>
+        <v>-4.559267425211544</v>
       </c>
       <c r="BS52" t="n">
-        <v>-13.40900768180216</v>
+        <v>-13.41476766822995</v>
       </c>
       <c r="BT52" t="b">
         <v>1</v>
@@ -12643,7 +12643,7 @@
         <v>-0.7524892122498517</v>
       </c>
       <c r="BS53" t="n">
-        <v>-10.10472871725758</v>
+        <v>-10.10473516918537</v>
       </c>
       <c r="BT53" t="b">
         <v>1</v>
@@ -14023,7 +14023,7 @@
         <v>-1.829967881255012</v>
       </c>
       <c r="BS59" t="n">
-        <v>-12.97565070002411</v>
+        <v>-12.97563698357254</v>
       </c>
       <c r="BT59" t="b">
         <v>1</v>
@@ -14254,7 +14254,7 @@
         <v>-2.380513347903379</v>
       </c>
       <c r="BS60" t="n">
-        <v>-39.31213242225636</v>
+        <v>-39.31213655317477</v>
       </c>
       <c r="BT60" t="b">
         <v>1</v>
@@ -14393,7 +14393,7 @@
         <v>8.789999999999999</v>
       </c>
       <c r="AQ61" t="n">
-        <v>8.34</v>
+        <v>8.33</v>
       </c>
       <c r="AR61" t="n">
         <v>14.13</v>
@@ -14414,13 +14414,13 @@
         <v>18.04999923706055</v>
       </c>
       <c r="AZ61" t="n">
-        <v>10.75</v>
+        <v>10.74</v>
       </c>
       <c r="BA61" t="n">
         <v>18.02</v>
       </c>
       <c r="BB61" t="n">
-        <v>28.55</v>
+        <v>28.59</v>
       </c>
       <c r="BC61" t="n">
         <v>30.08</v>
@@ -14429,7 +14429,7 @@
         <v>32.31</v>
       </c>
       <c r="BE61" t="n">
-        <v>19.1</v>
+        <v>19.11</v>
       </c>
       <c r="BF61" t="n">
         <v>18.02</v>
@@ -14441,10 +14441,10 @@
         <v>3</v>
       </c>
       <c r="BI61" t="n">
-        <v>-10.16</v>
+        <v>-10.15</v>
       </c>
       <c r="BJ61" t="n">
-        <v>5.84</v>
+        <v>5.89</v>
       </c>
       <c r="BK61" t="inlineStr">
         <is>
@@ -14475,7 +14475,7 @@
         <v>-4.752339322253274</v>
       </c>
       <c r="BS61" t="n">
-        <v>-15.01116941660103</v>
+        <v>-15.01472819110906</v>
       </c>
       <c r="BT61" t="b">
         <v>1</v>
@@ -15630,7 +15630,7 @@
         <v>-13.19352225208604</v>
       </c>
       <c r="BS66" t="n">
-        <v>-24.29702860875267</v>
+        <v>-24.29702155696503</v>
       </c>
       <c r="BT66" t="b">
         <v>1</v>
@@ -17257,7 +17257,7 @@
         <v>-4.332123386023334</v>
       </c>
       <c r="BS73" t="n">
-        <v>-23.36269571048517</v>
+        <v>-23.36268916509432</v>
       </c>
       <c r="BT73" t="b">
         <v>1</v>
@@ -19189,7 +19189,7 @@
         <v>-14.1804789183963</v>
       </c>
       <c r="BS8" t="n">
-        <v>-41.3906633420233</v>
+        <v>-41.39066698170934</v>
       </c>
       <c r="BT8" t="b">
         <v>1</v>
@@ -21953,7 +21953,7 @@
         <v>-3.049647471931205</v>
       </c>
       <c r="BS20" t="n">
-        <v>-21.08023573257425</v>
+        <v>-21.08022686888683</v>
       </c>
       <c r="BT20" t="b">
         <v>1</v>
@@ -22642,7 +22642,7 @@
         <v>-3.496970464635651</v>
       </c>
       <c r="BS23" t="n">
-        <v>-18.64655512043243</v>
+        <v>-18.64656395665553</v>
       </c>
       <c r="BT23" t="b">
         <v>1</v>
@@ -29201,7 +29201,7 @@
         <v>9.15</v>
       </c>
       <c r="AQ52" t="n">
-        <v>8.710000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="AR52" t="n">
         <v>14.13</v>
@@ -29222,13 +29222,13 @@
         <v>15.75</v>
       </c>
       <c r="AZ52" t="n">
-        <v>9.800000000000001</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="BA52" t="n">
-        <v>18.16</v>
+        <v>18.15</v>
       </c>
       <c r="BB52" t="n">
-        <v>31.55</v>
+        <v>31.57</v>
       </c>
       <c r="BC52" t="n">
         <v>30.13</v>
@@ -29237,22 +29237,22 @@
         <v>35.04</v>
       </c>
       <c r="BE52" t="n">
-        <v>19.84</v>
+        <v>19.83</v>
       </c>
       <c r="BF52" t="n">
-        <v>18.16</v>
+        <v>18.15</v>
       </c>
       <c r="BG52" t="n">
-        <v>16.35</v>
+        <v>16.33</v>
       </c>
       <c r="BH52" t="n">
         <v>3</v>
       </c>
       <c r="BI52" t="n">
-        <v>3.8</v>
+        <v>3.69</v>
       </c>
       <c r="BJ52" t="n">
-        <v>25.96</v>
+        <v>25.92</v>
       </c>
       <c r="BK52" t="inlineStr">
         <is>
@@ -29277,13 +29277,13 @@
         </is>
       </c>
       <c r="BQ52" t="n">
-        <v>16.50235748291016</v>
+        <v>16.50238800048828</v>
       </c>
       <c r="BR52" t="n">
-        <v>-4.559090928004061</v>
+        <v>-4.559267425211544</v>
       </c>
       <c r="BS52" t="n">
-        <v>-13.40900768180216</v>
+        <v>-13.41476766822995</v>
       </c>
       <c r="BT52" t="b">
         <v>1</v>
@@ -29514,7 +29514,7 @@
         <v>-0.7524892122498517</v>
       </c>
       <c r="BS53" t="n">
-        <v>-10.10472871725758</v>
+        <v>-10.10473516918537</v>
       </c>
       <c r="BT53" t="b">
         <v>1</v>
@@ -30894,7 +30894,7 @@
         <v>-1.829967881255012</v>
       </c>
       <c r="BS59" t="n">
-        <v>-12.97565070002411</v>
+        <v>-12.97563698357254</v>
       </c>
       <c r="BT59" t="b">
         <v>1</v>
@@ -31125,7 +31125,7 @@
         <v>-2.380513347903379</v>
       </c>
       <c r="BS60" t="n">
-        <v>-39.31213242225636</v>
+        <v>-39.31213655317477</v>
       </c>
       <c r="BT60" t="b">
         <v>1</v>
@@ -31264,7 +31264,7 @@
         <v>8.789999999999999</v>
       </c>
       <c r="AQ61" t="n">
-        <v>8.34</v>
+        <v>8.33</v>
       </c>
       <c r="AR61" t="n">
         <v>14.13</v>
@@ -31285,13 +31285,13 @@
         <v>18.04999923706055</v>
       </c>
       <c r="AZ61" t="n">
-        <v>10.75</v>
+        <v>10.74</v>
       </c>
       <c r="BA61" t="n">
         <v>18.02</v>
       </c>
       <c r="BB61" t="n">
-        <v>28.55</v>
+        <v>28.59</v>
       </c>
       <c r="BC61" t="n">
         <v>30.08</v>
@@ -31300,7 +31300,7 @@
         <v>32.31</v>
       </c>
       <c r="BE61" t="n">
-        <v>19.1</v>
+        <v>19.11</v>
       </c>
       <c r="BF61" t="n">
         <v>18.02</v>
@@ -31312,10 +31312,10 @@
         <v>3</v>
       </c>
       <c r="BI61" t="n">
-        <v>-10.16</v>
+        <v>-10.15</v>
       </c>
       <c r="BJ61" t="n">
-        <v>5.84</v>
+        <v>5.89</v>
       </c>
       <c r="BK61" t="inlineStr">
         <is>
@@ -31346,7 +31346,7 @@
         <v>-4.752339322253274</v>
       </c>
       <c r="BS61" t="n">
-        <v>-15.01116941660103</v>
+        <v>-15.01472819110906</v>
       </c>
       <c r="BT61" t="b">
         <v>1</v>
@@ -32501,7 +32501,7 @@
         <v>-13.19352225208604</v>
       </c>
       <c r="BS66" t="n">
-        <v>-24.29702860875267</v>
+        <v>-24.29702155696503</v>
       </c>
       <c r="BT66" t="b">
         <v>1</v>
@@ -34355,7 +34355,7 @@
         <v>-4.332123386023334</v>
       </c>
       <c r="BS74" t="n">
-        <v>-23.36269571048517</v>
+        <v>-23.36268916509432</v>
       </c>
       <c r="BT74" t="b">
         <v>1</v>
@@ -36394,7 +36394,7 @@
         <v>-2.956992813666715</v>
       </c>
       <c r="BS83" t="n">
-        <v>-50.64811100580535</v>
+        <v>-50.64811429232115</v>
       </c>
       <c r="BT83" t="b">
         <v>0</v>
@@ -37973,7 +37973,7 @@
         <v>-0.356291362225214</v>
       </c>
       <c r="BS90" t="n">
-        <v>-13.89556964471864</v>
+        <v>-13.89556104749984</v>
       </c>
       <c r="BT90" t="b">
         <v>0</v>
@@ -40659,7 +40659,7 @@
         <v>-0.1607677231829863</v>
       </c>
       <c r="BS102" t="n">
-        <v>-23.78160089072792</v>
+        <v>-23.78160993760151</v>
       </c>
       <c r="BT102" t="b">
         <v>0</v>
@@ -41230,7 +41230,7 @@
         <v>8.44</v>
       </c>
       <c r="AQ105" t="n">
-        <v>5.83</v>
+        <v>5.82</v>
       </c>
       <c r="AR105" t="n">
         <v>11.92</v>
@@ -41255,10 +41255,10 @@
         <v>7.960000038146973</v>
       </c>
       <c r="AZ105" t="n">
-        <v>3.32</v>
+        <v>3.31</v>
       </c>
       <c r="BA105" t="n">
-        <v>6.15</v>
+        <v>6.14</v>
       </c>
       <c r="BB105" t="n">
         <v>12.39</v>
@@ -41285,7 +41285,7 @@
         <v>32.65</v>
       </c>
       <c r="BJ105" t="n">
-        <v>33.46</v>
+        <v>33.43</v>
       </c>
       <c r="BK105" t="inlineStr">
         <is>
@@ -44836,7 +44836,7 @@
         <v>-5.657093049329509</v>
       </c>
       <c r="BS121" t="n">
-        <v>-16.25976554901378</v>
+        <v>-16.25975518349992</v>
       </c>
       <c r="BT121" t="b">
         <v>0</v>
@@ -45710,7 +45710,7 @@
         <v>-3.846150319251662</v>
       </c>
       <c r="BS125" t="n">
-        <v>-52.9902135681372</v>
+        <v>-52.99020827459822</v>
       </c>
       <c r="BT125" t="b">
         <v>0</v>

</xml_diff>